<commit_message>
Add extra options for ANATOMICAL_SITE
This matches the changes made in [MAV-4631](https://nhsd-jira.digital.nhs.uk/browse/MAV-4631)
</commit_message>
<xml_diff>
--- a/app/files/historical-vaccination-records-upload-template.xlsx
+++ b/app/files/historical-vaccination-records-upload-template.xlsx
@@ -1,11 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28723"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10315"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EB35E6F1-6FAC-43C6-A1E0-550FDF427592}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alistair/Downloads/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78D62948-FCB2-9349-AAE6-62CCB541E582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="240" yWindow="600" windowWidth="44700" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -237,9 +242,6 @@
     <t>Required only if VACCINE_GIVEN is omitted. Must be Y or N</t>
   </si>
   <si>
-    <t>Optional. It must be appropriate for the vaccine delivery method and be one of: left arm (lower position), left arm (upper position), left buttock, left thigh, left upper arm, nasal, right arm (lower position), right arm (upper position), right buttock, right thigh or right upper arm</t>
-  </si>
-  <si>
     <t>Required only if VACCINATED is N. Must be absent from school, already had elsewhere, did not attend, refused, unwell or vaccination contraindicated</t>
   </si>
   <si>
@@ -250,13 +252,16 @@
   </si>
   <si>
     <t>Required only if CARE_SETTING is 2. Must be the name of a community clinic location</t>
+  </si>
+  <si>
+    <t>Optional. It must be appropriate for the vaccine delivery method and be one of: left arm (lower position), left lower, left lower arm, left arm (upper position), left buttock, left thigh, left upper arm, nasal, right arm (lower position), right lower, right lower arm, right arm (upper position), right buttock, right thigh or right upper arm</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -268,7 +273,6 @@
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
-      <charset val="1"/>
     </font>
     <font>
       <b/>
@@ -674,34 +678,34 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Y2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="36.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="51.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="53.5703125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="53.28515625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="88.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="35.7109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="32.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="36.5" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="51.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="53.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="53.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="30.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="88.83203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="35.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="34.6640625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="32.5" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="77" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.42578125" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="46.5703125" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="51.5703125" customWidth="1"/>
-    <col min="17" max="17" width="228.85546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="123.42578125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.28515625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="43.5703125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="34.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="46.5" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="51.5" customWidth="1"/>
+    <col min="17" max="17" width="228.83203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="123.5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="8.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="43.5" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="34.83203125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="69" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="33.5" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="38" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="36.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -778,7 +782,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="29.25">
+    <row r="2" spans="1:25" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>25</v>
       </c>
@@ -828,22 +832,22 @@
         <v>39</v>
       </c>
       <c r="Q2" t="s">
+        <v>44</v>
+      </c>
+      <c r="R2" s="6" t="s">
         <v>40</v>
-      </c>
-      <c r="R2" s="6" t="s">
-        <v>41</v>
       </c>
       <c r="S2" t="s">
         <v>37</v>
       </c>
       <c r="T2" t="s">
+        <v>41</v>
+      </c>
+      <c r="U2" t="s">
         <v>42</v>
       </c>
-      <c r="U2" t="s">
+      <c r="V2" s="6" t="s">
         <v>43</v>
-      </c>
-      <c r="V2" s="6" t="s">
-        <v>44</v>
       </c>
       <c r="W2" t="s">
         <v>37</v>
@@ -861,15 +865,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FDE5462C73D2BC4498C7AF3E5E39BA62" ma:contentTypeVersion="55" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fdfcab40565e92f5d919ffbdffa6c15b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="80d05917-893e-4a06-bb39-47099b578ffd" xmlns:ns3="754dda3c-967d-4b24-9bc2-1cc61ceab4bc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="da7f0a503997aad593060802265a0e90" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -1161,6 +1156,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1181,13 +1185,41 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1612B58E-756E-4988-BA1E-2D26BC726FEA}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F680FFE-A4FA-4E53-8492-3F05C00224BE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="80d05917-893e-4a06-bb39-47099b578ffd"/>
+    <ds:schemaRef ds:uri="754dda3c-967d-4b24-9bc2-1cc61ceab4bc"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F680FFE-A4FA-4E53-8492-3F05C00224BE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1612B58E-756E-4988-BA1E-2D26BC726FEA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A951C6D7-CFFA-41B9-8357-81D1BE5BF461}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A951C6D7-CFFA-41B9-8357-81D1BE5BF461}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="80d05917-893e-4a06-bb39-47099b578ffd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="754dda3c-967d-4b24-9bc2-1cc61ceab4bc"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Add MMR and Flu vaccines to uplaod template
Updates hint text
</commit_message>
<xml_diff>
--- a/app/files/historical-vaccination-records-upload-template.xlsx
+++ b/app/files/historical-vaccination-records-upload-template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alistair/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lakshmimurugappan/Documents/Mavis/UserGuide/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78D62948-FCB2-9349-AAE6-62CCB541E582}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E73A4C28-7B6C-3D4D-9678-262C3D66613A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="600" windowWidth="44700" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -179,25 +179,6 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color rgb="FF242424"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t>Required</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF242424"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t>. Must be HPV, ACWYX4, MenACWY, 3-in-1, or Td/IPV</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
@@ -230,9 +211,6 @@
     <t>Optional. Must use HH:MM:SS format</t>
   </si>
   <si>
-    <t>Optional. Must be Cervarix, Gardasil, Gardasil9, MenQuadfi, Menveo, Nimenrix, or Revaxis</t>
-  </si>
-  <si>
     <t>Optional</t>
   </si>
   <si>
@@ -255,13 +233,19 @@
   </si>
   <si>
     <t>Optional. It must be appropriate for the vaccine delivery method and be one of: left arm (lower position), left lower, left lower arm, left arm (upper position), left buttock, left thigh, left upper arm, nasal, right arm (lower position), right lower, right lower arm, right arm (upper position), right buttock, right thigh or right upper arm</t>
+  </si>
+  <si>
+    <t>Required. Must be Flu, HPV, MMR, MMRV, ACWYX4, MenACWY, 3-in-1, or Td/IPV</t>
+  </si>
+  <si>
+    <t>Optional. Must be Sequirus Cell-based Trivalent, AstraZeneca Fluenz, Sanofi Vaxigrip, Viatris, Cervarix, Gardasil, Gardasil9, MenQuadfi, Menveo, Nimenrix, Priorix, VaxPro, ProQuad, Priorix-Tetra or Revaxis</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -289,11 +273,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FF242424"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
@@ -335,14 +314,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -792,71 +771,71 @@
       <c r="C2" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="7" t="s">
+      <c r="D2" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="E2" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="7" t="s">
+        <v>43</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="G2" s="3" t="s">
+      <c r="H2" t="s">
         <v>30</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>31</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>32</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>33</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="L2" s="1" t="s">
+      <c r="M2" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="N2" t="s">
         <v>35</v>
       </c>
-      <c r="M2" s="1" t="s">
+      <c r="O2" t="s">
         <v>36</v>
       </c>
-      <c r="N2" t="s">
+      <c r="P2" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="O2" t="s">
+      <c r="Q2" t="s">
+        <v>42</v>
+      </c>
+      <c r="R2" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="P2" s="6" t="s">
+      <c r="S2" t="s">
+        <v>35</v>
+      </c>
+      <c r="T2" t="s">
         <v>39</v>
       </c>
-      <c r="Q2" t="s">
-        <v>44</v>
-      </c>
-      <c r="R2" s="6" t="s">
+      <c r="U2" t="s">
         <v>40</v>
       </c>
-      <c r="S2" t="s">
-        <v>37</v>
-      </c>
-      <c r="T2" t="s">
+      <c r="V2" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="U2" t="s">
-        <v>42</v>
-      </c>
-      <c r="V2" s="6" t="s">
-        <v>43</v>
-      </c>
       <c r="W2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="X2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="Y2" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -865,6 +844,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FDE5462C73D2BC4498C7AF3E5E39BA62" ma:contentTypeVersion="55" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="fdfcab40565e92f5d919ffbdffa6c15b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns2="80d05917-893e-4a06-bb39-47099b578ffd" xmlns:ns3="754dda3c-967d-4b24-9bc2-1cc61ceab4bc" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="da7f0a503997aad593060802265a0e90" ns1:_="" ns2:_="" ns3:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -1156,15 +1144,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -1185,6 +1164,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1612B58E-756E-4988-BA1E-2D26BC726FEA}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F680FFE-A4FA-4E53-8492-3F05C00224BE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1204,14 +1191,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1612B58E-756E-4988-BA1E-2D26BC726FEA}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A951C6D7-CFFA-41B9-8357-81D1BE5BF461}">
   <ds:schemaRefs>

</xml_diff>

<commit_message>
Update hint text for immunisation import template
</commit_message>
<xml_diff>
--- a/app/files/historical-vaccination-records-upload-template.xlsx
+++ b/app/files/historical-vaccination-records-upload-template.xlsx
@@ -1,35 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10830"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lakshmimurugappan/Documents/Mavis/UserGuide/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E73A4C28-7B6C-3D4D-9678-262C3D66613A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="4"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="600" windowWidth="44700" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
+    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
@@ -38,255 +22,280 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
   <si>
-    <t>PERSON_FORENAME</t>
-  </si>
-  <si>
-    <t>PERSON_SURNAME</t>
-  </si>
-  <si>
-    <t>PERSON_DOB</t>
-  </si>
-  <si>
-    <t>PERSON_GENDER_CODE</t>
-  </si>
-  <si>
-    <t>PERSON_POSTCODE</t>
-  </si>
-  <si>
-    <t>PROGRAMME</t>
-  </si>
-  <si>
-    <t>DATE_OF_VACCINATION</t>
-  </si>
-  <si>
-    <t>ORGANISATION_CODE</t>
-  </si>
-  <si>
-    <t>SCHOOL_URN</t>
-  </si>
-  <si>
-    <t>SCHOOL_NAME</t>
-  </si>
-  <si>
-    <t>NHS_NUMBER</t>
-  </si>
-  <si>
-    <t>TIME_OF_VACCINATION</t>
-  </si>
-  <si>
-    <t>VACCINE_GIVEN</t>
-  </si>
-  <si>
-    <t>BATCH_NUMBER</t>
-  </si>
-  <si>
-    <t>BATCH_EXPIRY_DATE</t>
-  </si>
-  <si>
-    <t>VACCINATED</t>
-  </si>
-  <si>
-    <t>ANATOMICAL_SITE</t>
-  </si>
-  <si>
-    <t>REASON_NOT_VACCINATED</t>
-  </si>
-  <si>
-    <t>NOTES</t>
-  </si>
-  <si>
-    <t>DOSE_SEQUENCE</t>
-  </si>
-  <si>
-    <t>CARE_SETTING</t>
-  </si>
-  <si>
-    <t>CLINIC_NAME</t>
-  </si>
-  <si>
-    <t>PERFORMING_PROFESSIONAL_EMAIL</t>
-  </si>
-  <si>
-    <t>PERFORMING_PROFESSIONAL_FORENAME</t>
-  </si>
-  <si>
-    <t>PERFORMING_PROFESSIONAL_SURNAME</t>
-  </si>
-  <si>
-    <t>Required</t>
+    <t xml:space="preserve">PERSON_FORENAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERSON_SURNAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERSON_DOB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERSON_GENDER_CODE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERSON_POSTCODE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROGRAMME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATE_OF_VACCINATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORGANISATION_CODE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCHOOL_URN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCHOOL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NHS_NUMBER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TIME_OF_VACCINATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VACCINE_GIVEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BATCH_NUMBER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BATCH_EXPIRY_DATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VACCINATED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANATOMICAL_SITE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REASON_NOT_VACCINATED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOSE_SEQUENCE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CARE_SETTING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLINIC_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERFORMING_PROFESSIONAL_EMAIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERFORMING_PROFESSIONAL_FORENAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERFORMING_PROFESSIONAL_SURNAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required</t>
   </si>
   <si>
     <r>
       <rPr>
-        <b/>
+        <b val="true"/>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>Required</t>
+      <t xml:space="preserve">Required</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>. Must use either YYYYMMDD or DD/MM/YYYY</t>
+      <t xml:space="preserve">. Must use either YYYYMMDD or DD/MM/YYYY</t>
     </r>
   </si>
   <si>
     <r>
       <rPr>
-        <b/>
+        <b val="true"/>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>Required</t>
+      <t xml:space="preserve">Required</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>. Must be one of Not known, Male, Female, Not specified.</t>
+      <t xml:space="preserve">. Must be one of Not known, Male, Female, Not specified.</t>
     </r>
   </si>
   <si>
     <r>
       <rPr>
-        <b/>
+        <b val="true"/>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>Required</t>
+      <t xml:space="preserve">Required</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>. Must be a valid UK postcode</t>
+      <t xml:space="preserve">. Must be a valid UK postcode</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Required. Must be Flu, HPV, MMR, MMRV, ACWYX4, MenACWY, 3-in-1, or Td/IPV</t>
   </si>
   <si>
     <r>
       <rPr>
-        <b/>
+        <b val="true"/>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>Required</t>
+      <t xml:space="preserve">Required</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>. Must use either YYYYMMDD or DD/MM/YYYY format</t>
+      <t xml:space="preserve">. Must use either YYYYMMDD or DD/MM/YYYY format</t>
     </r>
   </si>
   <si>
-    <t>Optional. Must be a valid ODS code</t>
-  </si>
-  <si>
-    <t>Optional. Must be 6 digits and numeric. Use 888888 for school unknown and 999999 for homeschooled.</t>
-  </si>
-  <si>
-    <t>Required only if SCHOOL_URN is 888888</t>
-  </si>
-  <si>
-    <t>Optional. Must be 10 digits and numeric</t>
-  </si>
-  <si>
-    <t>Optional. Must use HH:MM:SS format</t>
-  </si>
-  <si>
-    <t>Optional</t>
-  </si>
-  <si>
-    <t>Optional. Must use either YYYYMMDD or DD/MM/YYYY</t>
-  </si>
-  <si>
-    <t>Required only if VACCINE_GIVEN is omitted. Must be Y or N</t>
-  </si>
-  <si>
-    <t>Required only if VACCINATED is N. Must be absent from school, already had elsewhere, did not attend, refused, unwell or vaccination contraindicated</t>
-  </si>
-  <si>
-    <t>Optional. Must be a number or 1B, 1P, 2B, 2P or 3P</t>
-  </si>
-  <si>
-    <t>Optional. Must be 1 (school) or 2 (clinic)</t>
-  </si>
-  <si>
-    <t>Required only if CARE_SETTING is 2. Must be the name of a community clinic location</t>
-  </si>
-  <si>
-    <t>Optional. It must be appropriate for the vaccine delivery method and be one of: left arm (lower position), left lower, left lower arm, left arm (upper position), left buttock, left thigh, left upper arm, nasal, right arm (lower position), right lower, right lower arm, right arm (upper position), right buttock, right thigh or right upper arm</t>
-  </si>
-  <si>
-    <t>Required. Must be Flu, HPV, MMR, MMRV, ACWYX4, MenACWY, 3-in-1, or Td/IPV</t>
-  </si>
-  <si>
-    <t>Optional. Must be Sequirus Cell-based Trivalent, AstraZeneca Fluenz, Sanofi Vaxigrip, Viatris, Cervarix, Gardasil, Gardasil9, MenQuadfi, Menveo, Nimenrix, Priorix, VaxPro, ProQuad, Priorix-Tetra or Revaxis</t>
+    <t xml:space="preserve">Optional. Must be a valid ODS code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Must be 6 digits and numeric. Use 888888 for school unknown and 999999 for homeschooled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required only if SCHOOL_URN is 888888</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Must be 10 digits and numeric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Must use HH:MM:SS format</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Must be Sequirus Cell-based Trivalent, AstraZeneca Fluenz, Sanofi Vaxigrip, Viatris, Cervarix, Gardasil, Gardasil9, MenQuadfi, Menveo, Nimenrix, Priorix, VaxPro, ProQuad, Priorix-Tetra or Revaxis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Must use either YYYYMMDD or DD/MM/YYYY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required only if VACCINE_GIVEN is omitted. Must be Y or N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. It must be appropriate for the vaccine delivery method and be one of: left arm (lower position), left lower, left lower arm, left arm (upper position), left buttock, left thigh, left upper arm, nasal, right arm (lower position), right lower, right lower arm, right arm (upper position), right buttock, right thigh or right upper arm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required only if VACCINATED is N. Must be absent from school, already had elsewhere, did not attend, refused, unwell or vaccination contraindicated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional, must be a number or 1B, 1P, 1st Scheduled Booster, 2B, 2P, 2nd Scheduled Booster or 3P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Must be 1 (school) or 2 (clinic)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required only if CARE_SETTING is 2. Must be the name of a community clinic location</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="General"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Aptos Narrow"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF242424"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -298,7 +307,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
@@ -306,48 +315,137 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+  <cellXfs count="6">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF242424"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -382,153 +480,55 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="020F0302020204030204"/>
+        <a:latin typeface="Aptos Display" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme>
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
                 <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
                 <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
                 <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
                 <a:lumMod val="102000"/>
                 <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
                 <a:lumMod val="100000"/>
                 <a:shade val="100000"/>
               </a:schemeClr>
@@ -536,33 +536,24 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
                 <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
@@ -575,13 +566,7 @@
           <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -591,15 +576,13 @@
         <a:solidFill>
           <a:schemeClr val="phClr">
             <a:tint val="95000"/>
-            <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
               </a:schemeClr>
@@ -607,7 +590,6 @@
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
               </a:schemeClr>
@@ -615,231 +597,213 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="63000"/>
-                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:Y2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="36.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="51.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="53.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="53.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="88.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="32.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="77" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="46.5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="51.5" customWidth="1"/>
-    <col min="17" max="17" width="228.83203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="123.5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="43.5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="34.83203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="69" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="33.5" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="38" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="36.83203125" bestFit="1" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="36.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="51.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="53.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="53.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="88.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="35.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="34.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="32.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="15.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="46.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="51.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="228.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="123.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="8.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="81.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="34.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="33.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="36.83"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="0" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="32" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="N2" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="O2" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="S2" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="T2" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="U2" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="H2" t="s">
-        <v>30</v>
-      </c>
-      <c r="I2" t="s">
-        <v>31</v>
-      </c>
-      <c r="J2" t="s">
-        <v>32</v>
-      </c>
-      <c r="K2" t="s">
-        <v>33</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="M2" s="1" t="s">
+      <c r="V2" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="N2" t="s">
-        <v>35</v>
-      </c>
-      <c r="O2" t="s">
-        <v>36</v>
-      </c>
-      <c r="P2" s="5" t="s">
+      <c r="W2" s="0" t="s">
         <v>37</v>
       </c>
-      <c r="Q2" t="s">
-        <v>42</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="S2" t="s">
-        <v>35</v>
-      </c>
-      <c r="T2" t="s">
-        <v>39</v>
-      </c>
-      <c r="U2" t="s">
-        <v>40</v>
-      </c>
-      <c r="V2" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="W2" t="s">
-        <v>35</v>
-      </c>
-      <c r="X2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>35</v>
+      <c r="X2" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y2" s="0" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Update hint text for immunisation import template (#228)
</commit_message>
<xml_diff>
--- a/app/files/historical-vaccination-records-upload-template.xlsx
+++ b/app/files/historical-vaccination-records-upload-template.xlsx
@@ -1,35 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10830"/>
-  <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lakshmimurugappan/Documents/Mavis/UserGuide/"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E73A4C28-7B6C-3D4D-9678-262C3D66613A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+  <fileVersion appName="Calc" lowestEdited="4"/>
+  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
+  <workbookProtection/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="600" windowWidth="44700" windowHeight="15680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
+    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
@@ -38,255 +22,280 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="45">
   <si>
-    <t>PERSON_FORENAME</t>
-  </si>
-  <si>
-    <t>PERSON_SURNAME</t>
-  </si>
-  <si>
-    <t>PERSON_DOB</t>
-  </si>
-  <si>
-    <t>PERSON_GENDER_CODE</t>
-  </si>
-  <si>
-    <t>PERSON_POSTCODE</t>
-  </si>
-  <si>
-    <t>PROGRAMME</t>
-  </si>
-  <si>
-    <t>DATE_OF_VACCINATION</t>
-  </si>
-  <si>
-    <t>ORGANISATION_CODE</t>
-  </si>
-  <si>
-    <t>SCHOOL_URN</t>
-  </si>
-  <si>
-    <t>SCHOOL_NAME</t>
-  </si>
-  <si>
-    <t>NHS_NUMBER</t>
-  </si>
-  <si>
-    <t>TIME_OF_VACCINATION</t>
-  </si>
-  <si>
-    <t>VACCINE_GIVEN</t>
-  </si>
-  <si>
-    <t>BATCH_NUMBER</t>
-  </si>
-  <si>
-    <t>BATCH_EXPIRY_DATE</t>
-  </si>
-  <si>
-    <t>VACCINATED</t>
-  </si>
-  <si>
-    <t>ANATOMICAL_SITE</t>
-  </si>
-  <si>
-    <t>REASON_NOT_VACCINATED</t>
-  </si>
-  <si>
-    <t>NOTES</t>
-  </si>
-  <si>
-    <t>DOSE_SEQUENCE</t>
-  </si>
-  <si>
-    <t>CARE_SETTING</t>
-  </si>
-  <si>
-    <t>CLINIC_NAME</t>
-  </si>
-  <si>
-    <t>PERFORMING_PROFESSIONAL_EMAIL</t>
-  </si>
-  <si>
-    <t>PERFORMING_PROFESSIONAL_FORENAME</t>
-  </si>
-  <si>
-    <t>PERFORMING_PROFESSIONAL_SURNAME</t>
-  </si>
-  <si>
-    <t>Required</t>
+    <t xml:space="preserve">PERSON_FORENAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERSON_SURNAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERSON_DOB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERSON_GENDER_CODE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERSON_POSTCODE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PROGRAMME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATE_OF_VACCINATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ORGANISATION_CODE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCHOOL_URN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SCHOOL_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NHS_NUMBER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TIME_OF_VACCINATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VACCINE_GIVEN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BATCH_NUMBER</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BATCH_EXPIRY_DATE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VACCINATED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ANATOMICAL_SITE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REASON_NOT_VACCINATED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NOTES</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOSE_SEQUENCE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CARE_SETTING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLINIC_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERFORMING_PROFESSIONAL_EMAIL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERFORMING_PROFESSIONAL_FORENAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PERFORMING_PROFESSIONAL_SURNAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required</t>
   </si>
   <si>
     <r>
       <rPr>
-        <b/>
+        <b val="true"/>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>Required</t>
+      <t xml:space="preserve">Required</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>. Must use either YYYYMMDD or DD/MM/YYYY</t>
+      <t xml:space="preserve">. Must use either YYYYMMDD or DD/MM/YYYY</t>
     </r>
   </si>
   <si>
     <r>
       <rPr>
-        <b/>
+        <b val="true"/>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>Required</t>
+      <t xml:space="preserve">Required</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>. Must be one of Not known, Male, Female, Not specified.</t>
+      <t xml:space="preserve">. Must be one of Not known, Male, Female, Not specified.</t>
     </r>
   </si>
   <si>
     <r>
       <rPr>
-        <b/>
+        <b val="true"/>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>Required</t>
+      <t xml:space="preserve">Required</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>. Must be a valid UK postcode</t>
+      <t xml:space="preserve">. Must be a valid UK postcode</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">Required. Must be Flu, HPV, MMR, MMRV, ACWYX4, MenACWY, 3-in-1, or Td/IPV</t>
   </si>
   <si>
     <r>
       <rPr>
-        <b/>
+        <b val="true"/>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>Required</t>
+      <t xml:space="preserve">Required</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <scheme val="minor"/>
+        <family val="0"/>
+        <charset val="1"/>
       </rPr>
-      <t>. Must use either YYYYMMDD or DD/MM/YYYY format</t>
+      <t xml:space="preserve">. Must use either YYYYMMDD or DD/MM/YYYY format</t>
     </r>
   </si>
   <si>
-    <t>Optional. Must be a valid ODS code</t>
-  </si>
-  <si>
-    <t>Optional. Must be 6 digits and numeric. Use 888888 for school unknown and 999999 for homeschooled.</t>
-  </si>
-  <si>
-    <t>Required only if SCHOOL_URN is 888888</t>
-  </si>
-  <si>
-    <t>Optional. Must be 10 digits and numeric</t>
-  </si>
-  <si>
-    <t>Optional. Must use HH:MM:SS format</t>
-  </si>
-  <si>
-    <t>Optional</t>
-  </si>
-  <si>
-    <t>Optional. Must use either YYYYMMDD or DD/MM/YYYY</t>
-  </si>
-  <si>
-    <t>Required only if VACCINE_GIVEN is omitted. Must be Y or N</t>
-  </si>
-  <si>
-    <t>Required only if VACCINATED is N. Must be absent from school, already had elsewhere, did not attend, refused, unwell or vaccination contraindicated</t>
-  </si>
-  <si>
-    <t>Optional. Must be a number or 1B, 1P, 2B, 2P or 3P</t>
-  </si>
-  <si>
-    <t>Optional. Must be 1 (school) or 2 (clinic)</t>
-  </si>
-  <si>
-    <t>Required only if CARE_SETTING is 2. Must be the name of a community clinic location</t>
-  </si>
-  <si>
-    <t>Optional. It must be appropriate for the vaccine delivery method and be one of: left arm (lower position), left lower, left lower arm, left arm (upper position), left buttock, left thigh, left upper arm, nasal, right arm (lower position), right lower, right lower arm, right arm (upper position), right buttock, right thigh or right upper arm</t>
-  </si>
-  <si>
-    <t>Required. Must be Flu, HPV, MMR, MMRV, ACWYX4, MenACWY, 3-in-1, or Td/IPV</t>
-  </si>
-  <si>
-    <t>Optional. Must be Sequirus Cell-based Trivalent, AstraZeneca Fluenz, Sanofi Vaxigrip, Viatris, Cervarix, Gardasil, Gardasil9, MenQuadfi, Menveo, Nimenrix, Priorix, VaxPro, ProQuad, Priorix-Tetra or Revaxis</t>
+    <t xml:space="preserve">Optional. Must be a valid ODS code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Must be 6 digits and numeric. Use 888888 for school unknown and 999999 for homeschooled.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required only if SCHOOL_URN is 888888</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Must be 10 digits and numeric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Must use HH:MM:SS format</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Must be Sequirus Cell-based Trivalent, AstraZeneca Fluenz, Sanofi Vaxigrip, Viatris, Cervarix, Gardasil, Gardasil9, MenQuadfi, Menveo, Nimenrix, Priorix, VaxPro, ProQuad, Priorix-Tetra or Revaxis</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Must use either YYYYMMDD or DD/MM/YYYY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required only if VACCINE_GIVEN is omitted. Must be Y or N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. It must be appropriate for the vaccine delivery method and be one of: left arm (lower position), left lower, left lower arm, left arm (upper position), left buttock, left thigh, left upper arm, nasal, right arm (lower position), right lower, right lower arm, right arm (upper position), right buttock, right thigh or right upper arm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required only if VACCINATED is N. Must be absent from school, already had elsewhere, did not attend, refused, unwell or vaccination contraindicated</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional, must be a number or 1B, 1P, 1st Scheduled Booster, 2B, 2P, 2nd Scheduled Booster or 3P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional. Must be 1 (school) or 2 (clinic)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Required only if CARE_SETTING is 2. Must be the name of a community clinic location</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="General"/>
+  </numFmts>
+  <fonts count="8">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
-      <scheme val="minor"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="11"/>
+      <color rgb="FF242424"/>
+      <name val="Aptos Narrow"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FF242424"/>
       <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF242424"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Aptos Narrow"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -298,7 +307,7 @@
     </fill>
   </fills>
   <borders count="1">
-    <border>
+    <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
       <top/>
@@ -306,48 +315,137 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  <cellStyleXfs count="20">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
+  <cellXfs count="6">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="15" builtinId="3"/>
+    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
+    <cellStyle name="Currency" xfId="17" builtinId="4"/>
+    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
+    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleMedium9"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="FF000000"/>
+      <rgbColor rgb="FFFFFFFF"/>
+      <rgbColor rgb="FFFF0000"/>
+      <rgbColor rgb="FF00FF00"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008000"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FF808000"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FF808080"/>
+      <rgbColor rgb="FF9999FF"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FFFFFFCC"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FF660066"/>
+      <rgbColor rgb="FFFF8080"/>
+      <rgbColor rgb="FF0066CC"/>
+      <rgbColor rgb="FFCCCCFF"/>
+      <rgbColor rgb="FF000080"/>
+      <rgbColor rgb="FFFF00FF"/>
+      <rgbColor rgb="FFFFFF00"/>
+      <rgbColor rgb="FF00FFFF"/>
+      <rgbColor rgb="FF800080"/>
+      <rgbColor rgb="FF800000"/>
+      <rgbColor rgb="FF008080"/>
+      <rgbColor rgb="FF0000FF"/>
+      <rgbColor rgb="FF00CCFF"/>
+      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FF99CCFF"/>
+      <rgbColor rgb="FFFF99CC"/>
+      <rgbColor rgb="FFCC99FF"/>
+      <rgbColor rgb="FFFFCC99"/>
+      <rgbColor rgb="FF3366FF"/>
+      <rgbColor rgb="FF33CCCC"/>
+      <rgbColor rgb="FF99CC00"/>
+      <rgbColor rgb="FFFFCC00"/>
+      <rgbColor rgb="FFFF9900"/>
+      <rgbColor rgb="FFFF6600"/>
+      <rgbColor rgb="FF666699"/>
+      <rgbColor rgb="FF969696"/>
+      <rgbColor rgb="FF003366"/>
+      <rgbColor rgb="FF339966"/>
+      <rgbColor rgb="FF003300"/>
+      <rgbColor rgb="FF333300"/>
+      <rgbColor rgb="FF993300"/>
+      <rgbColor rgb="FF993366"/>
+      <rgbColor rgb="FF333399"/>
+      <rgbColor rgb="FF242424"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
-        <a:sysClr val="windowText" lastClr="000000"/>
+        <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:sysClr val="window" lastClr="FFFFFF"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
         <a:srgbClr val="0E2841"/>
@@ -382,153 +480,55 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="020F0302020204030204"/>
+        <a:latin typeface="Aptos Display" panose="020F0302020204030204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック Light"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线 Light"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Times New Roman"/>
-        <a:font script="Hebr" typeface="Times New Roman"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="MoolBoran"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Times New Roman"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow" panose="02110004020202020204" pitchFamily="0" charset="1"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="游ゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="等线"/>
-        <a:font script="Hant" typeface="新細明體"/>
-        <a:font script="Arab" typeface="Arial"/>
-        <a:font script="Hebr" typeface="Arial"/>
-        <a:font script="Thai" typeface="Tahoma"/>
-        <a:font script="Ethi" typeface="Nyala"/>
-        <a:font script="Beng" typeface="Vrinda"/>
-        <a:font script="Gujr" typeface="Shruti"/>
-        <a:font script="Khmr" typeface="DaunPenh"/>
-        <a:font script="Knda" typeface="Tunga"/>
-        <a:font script="Guru" typeface="Raavi"/>
-        <a:font script="Cans" typeface="Euphemia"/>
-        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
-        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
-        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
-        <a:font script="Thaa" typeface="MV Boli"/>
-        <a:font script="Deva" typeface="Mangal"/>
-        <a:font script="Telu" typeface="Gautami"/>
-        <a:font script="Taml" typeface="Latha"/>
-        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
-        <a:font script="Orya" typeface="Kalinga"/>
-        <a:font script="Mlym" typeface="Kartika"/>
-        <a:font script="Laoo" typeface="DokChampa"/>
-        <a:font script="Sinh" typeface="Iskoola Pota"/>
-        <a:font script="Mong" typeface="Mongolian Baiti"/>
-        <a:font script="Viet" typeface="Arial"/>
-        <a:font script="Uigh" typeface="Microsoft Uighur"/>
-        <a:font script="Geor" typeface="Sylfaen"/>
-        <a:font script="Armn" typeface="Arial"/>
-        <a:font script="Bugi" typeface="Leelawadee UI"/>
-        <a:font script="Bopo" typeface="Microsoft JhengHei"/>
-        <a:font script="Java" typeface="Javanese Text"/>
-        <a:font script="Lisu" typeface="Segoe UI"/>
-        <a:font script="Mymr" typeface="Myanmar Text"/>
-        <a:font script="Nkoo" typeface="Ebrima"/>
-        <a:font script="Olck" typeface="Nirmala UI"/>
-        <a:font script="Osma" typeface="Ebrima"/>
-        <a:font script="Phag" typeface="Phagspa"/>
-        <a:font script="Syrn" typeface="Estrangelo Edessa"/>
-        <a:font script="Syrj" typeface="Estrangelo Edessa"/>
-        <a:font script="Syre" typeface="Estrangelo Edessa"/>
-        <a:font script="Sora" typeface="Nirmala UI"/>
-        <a:font script="Tale" typeface="Microsoft Tai Le"/>
-        <a:font script="Talu" typeface="Microsoft New Tai Lue"/>
-        <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme>
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
                 <a:tint val="67000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
                 <a:tint val="73000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
                 <a:tint val="81000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
                 <a:lumMod val="102000"/>
                 <a:tint val="94000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
                 <a:lumMod val="100000"/>
                 <a:shade val="100000"/>
               </a:schemeClr>
@@ -536,33 +536,24 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
                 <a:shade val="78000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
           <a:prstDash val="solid"/>
           <a:miter lim="800000"/>
         </a:ln>
@@ -575,13 +566,7 @@
           <a:effectLst/>
         </a:effectStyle>
         <a:effectStyle>
-          <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
-              <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
-              </a:srgbClr>
-            </a:outerShdw>
-          </a:effectLst>
+          <a:effectLst/>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
@@ -591,15 +576,13 @@
         <a:solidFill>
           <a:schemeClr val="phClr">
             <a:tint val="95000"/>
-            <a:satMod val="170000"/>
           </a:schemeClr>
         </a:solidFill>
-        <a:gradFill rotWithShape="1">
+        <a:gradFill>
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
                 <a:tint val="93000"/>
-                <a:satMod val="150000"/>
                 <a:shade val="98000"/>
                 <a:lumMod val="102000"/>
               </a:schemeClr>
@@ -607,7 +590,6 @@
             <a:gs pos="50000">
               <a:schemeClr val="phClr">
                 <a:tint val="98000"/>
-                <a:satMod val="130000"/>
                 <a:shade val="90000"/>
                 <a:lumMod val="103000"/>
               </a:schemeClr>
@@ -615,231 +597,213 @@
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
                 <a:shade val="63000"/>
-                <a:satMod val="120000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
           <a:lin ang="5400000" scaled="0"/>
+          <a:tileRect l="0" t="0" r="0" b="0"/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
-  <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
   <dimension ref="A1:Y2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="3" max="3" width="28" customWidth="1"/>
-    <col min="4" max="4" width="36.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="51.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="53.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="53.33203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="30.6640625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="88.83203125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="35.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="34.6640625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="32.5" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="77" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="46.5" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="51.5" customWidth="1"/>
-    <col min="17" max="17" width="228.83203125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="123.5" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="8.33203125" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="43.5" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="34.83203125" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="69" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="33.5" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="38" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="36.83203125" bestFit="1" customWidth="1"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="28"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="36.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="51.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="53.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="53.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="30.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="88.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="35.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="34.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="32.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="13" min="13" style="0" width="77"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="14" min="14" style="0" width="15.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="15" min="15" style="0" width="46.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16" min="16" style="0" width="51.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="17" min="17" style="0" width="228.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="18" min="18" style="0" width="123.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="19" min="19" style="0" width="8.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="20" style="0" width="81.23"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="21" style="0" width="34.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="22" min="22" style="0" width="69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="23" min="23" style="0" width="33.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="24" min="24" style="0" width="38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="25" min="25" style="0" width="36.83"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="0" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="0" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="0" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="0" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="0" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="0" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="0" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="0" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="0" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="0" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="0" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="0" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="0" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="0" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="0" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="0" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="0" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="0" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="0" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="0" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="0" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="0" t="s">
         <v>22</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="0" t="s">
         <v>23</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="0" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25" ht="32" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+    <row r="2" customFormat="false" ht="30.1" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="7" t="s">
+      <c r="F2" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H2" s="0" t="s">
+        <v>31</v>
+      </c>
+      <c r="I2" s="0" t="s">
+        <v>32</v>
+      </c>
+      <c r="J2" s="0" t="s">
+        <v>33</v>
+      </c>
+      <c r="K2" s="0" t="s">
+        <v>34</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="M2" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="N2" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="O2" s="0" t="s">
+        <v>38</v>
+      </c>
+      <c r="P2" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="Q2" s="0" t="s">
+        <v>40</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="S2" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="T2" s="0" t="s">
+        <v>42</v>
+      </c>
+      <c r="U2" s="0" t="s">
         <v>43</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="H2" t="s">
-        <v>30</v>
-      </c>
-      <c r="I2" t="s">
-        <v>31</v>
-      </c>
-      <c r="J2" t="s">
-        <v>32</v>
-      </c>
-      <c r="K2" t="s">
-        <v>33</v>
-      </c>
-      <c r="L2" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="M2" s="1" t="s">
+      <c r="V2" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="N2" t="s">
-        <v>35</v>
-      </c>
-      <c r="O2" t="s">
-        <v>36</v>
-      </c>
-      <c r="P2" s="5" t="s">
+      <c r="W2" s="0" t="s">
         <v>37</v>
       </c>
-      <c r="Q2" t="s">
-        <v>42</v>
-      </c>
-      <c r="R2" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="S2" t="s">
-        <v>35</v>
-      </c>
-      <c r="T2" t="s">
-        <v>39</v>
-      </c>
-      <c r="U2" t="s">
-        <v>40</v>
-      </c>
-      <c r="V2" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="W2" t="s">
-        <v>35</v>
-      </c>
-      <c r="X2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>35</v>
+      <c r="X2" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y2" s="0" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 

</xml_diff>